<commit_message>
feat: implement Milestone 3 Interview Assistance, ATS Integration, and Admin Management
- Role-Specific Interview Question Generator with technical & behavioral templates for 10+ engineering roles.

- AI Interview Simulation Chatbot with real-time scoring (Clarity, Relevance, Overall) and automatic candidate status sync.

- ATS REST API endpoints (/ats/add_candidate, /ats/list_candidates, /ats/update_status) and live status tracking widget.

- Main Admin capabilities to edit candidate Current Role and Total Experience Years across views with real-time match score recalculation.

- Enhanced candidate search filter, custom skills edit options, and batch evaluation pipeline outputs.
</commit_message>
<xml_diff>
--- a/matching_results.xlsx
+++ b/matching_results.xlsx
@@ -425,31 +425,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Candidate</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Job Title</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Skill Match (%)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Hiring Score (%)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Benchmark Status</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Alert</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Matched Skills</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Missing Skills</t>
         </is>
@@ -458,146 +478,379 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Sarah Johnson</t>
+          <t>#1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>76</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Python, TensorFlow, SQL</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Kubernetes, AWS SageMaker</t>
-        </is>
-      </c>
+          <t>Alex Chen</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Backend Java Specialist</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>100</v>
+      </c>
+      <c r="E2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>QUALIFIED (100.0% &gt;= 85%)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>None (Meets &gt;=85% Target)</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Docker, Java, SQL</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>#2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>Sarah Johnson</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Backend Developer</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>40</v>
-      </c>
-      <c r="D3" t="inlineStr">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Backend Java Specialist</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>33.33</v>
+      </c>
+      <c r="E3" t="n">
+        <v>56.25</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>ALERT (33.33% &lt; 85%)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>ALERT: Skill match 33.33% is below 85% requirement. Upskilling recommended in: Docker, Java</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>SQL</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>AWS, Java, Spring</t>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Docker, Java</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>David Lee</t>
+          <t>#3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>37</v>
-      </c>
-      <c r="D4" t="inlineStr">
+          <t>Emily Rodriguez</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Backend Java Specialist</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>33.33</v>
+      </c>
+      <c r="E4" t="n">
+        <v>56.25</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>ALERT (33.33% &lt; 85%)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>ALERT: Skill match 33.33% is below 85% requirement. Upskilling recommended in: Docker, Java</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>SQL</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Python, TensorFlow, Kubernetes, AWS SageMaker</t>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Docker, Java</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>David Lee</t>
+          <t>#1</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Backend Developer</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>100</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>SQL, AWS, Java, Spring</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
+          <t>Alex Chen</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>DevOps &amp; Cloud Engineer</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>75</v>
+      </c>
+      <c r="E5" t="n">
+        <v>78.75</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>ALERT (75.0% &lt; 85%)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>ALERT: Skill match 75.0% is below 85% requirement. Upskilling recommended in: AWS</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Docker, Kubernetes, Python</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>AWS</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Priya Sharma</t>
+          <t>#2</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>69.75</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Python, SQL, Kubernetes</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>TensorFlow, AWS SageMaker</t>
+          <t>Emily Rodriguez</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>DevOps &amp; Cloud Engineer</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>50</v>
+      </c>
+      <c r="E6" t="n">
+        <v>66.25</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>ALERT (50.0% &lt; 85%)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>ALERT: Skill match 50.0% is below 85% requirement. Upskilling recommended in: Docker, AWS</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Kubernetes, Python</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Docker, AWS</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Priya Sharma</t>
+          <t>#3</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Backend Developer</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>55</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>SQL, AWS</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Java, Spring</t>
+          <t>Sarah Johnson</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>DevOps &amp; Cloud Engineer</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>25</v>
+      </c>
+      <c r="E7" t="n">
+        <v>51.25</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>ALERT (25.0% &lt; 85%)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>ALERT: Skill match 25.0% is below 85% requirement. Upskilling recommended in: Docker, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Docker, Kubernetes, AWS</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>#1</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Emily Rodriguez</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Senior Machine Learning Engineer</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>100</v>
+      </c>
+      <c r="E8" t="n">
+        <v>100</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>QUALIFIED (100.0% &gt;= 85%)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>None (Meets &gt;=85% Target)</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>AWS SageMaker, Python, TensorFlow, Kubernetes, SQL</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>#2</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Sarah Johnson</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Senior Machine Learning Engineer</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>60</v>
+      </c>
+      <c r="E9" t="n">
+        <v>76</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>ALERT (60.0% &lt; 85%)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>ALERT: Skill match 60.0% is below 85% requirement. Upskilling recommended in: Kubernetes, AWS SageMaker</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>SQL, Python, TensorFlow</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Kubernetes, AWS SageMaker</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>#3</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Alex Chen</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Senior Machine Learning Engineer</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>60</v>
+      </c>
+      <c r="E10" t="n">
+        <v>66</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>ALERT (60.0% &lt; 85%)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>ALERT: Skill match 60.0% is below 85% requirement. Upskilling recommended in: AWS SageMaker, TensorFlow</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Kubernetes, Python, SQL</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>AWS SageMaker, TensorFlow</t>
         </is>
       </c>
     </row>

</xml_diff>